<commit_message>
20260501_190000 - add shareFile to all modules + MainActivity JsInterface
shareFile(base64Data, fileName, mimeType) saves to cache and triggers
Android Intent.ACTION_SEND chooser for sharing generated reports.
Modules updated: busbar-check, battery-test, capacitor-check,
elevator-handrail-fault (2 reports), power-room-monthly (PDF)
</commit_message>
<xml_diff>
--- a/app/build/intermediates/assets/debug/templates/busbar_template.xlsx
+++ b/app/build/intermediates/assets/debug/templates/busbar_template.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="54">
   <si>
     <t>供电母排检查测温记录表</t>
   </si>
@@ -186,6 +186,45 @@
       </rPr>
       <t xml:space="preserve">                                                                                               </t>
     </r>
+  </si>
+  <si>
+    <t>29层</t>
+  </si>
+  <si>
+    <t>28层</t>
+  </si>
+  <si>
+    <t>27层</t>
+  </si>
+  <si>
+    <t>26层</t>
+  </si>
+  <si>
+    <t>25层</t>
+  </si>
+  <si>
+    <t>23层</t>
+  </si>
+  <si>
+    <t>22层</t>
+  </si>
+  <si>
+    <t>21层</t>
+  </si>
+  <si>
+    <t>20层</t>
+  </si>
+  <si>
+    <t>19层</t>
+  </si>
+  <si>
+    <t>18层</t>
+  </si>
+  <si>
+    <t>17层</t>
+  </si>
+  <si>
+    <t>16层</t>
   </si>
 </sst>
 </file>
@@ -1368,7 +1407,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="16" width="13.875" style="1" customWidth="1"/>
@@ -1930,28 +1969,116 @@
       </c>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
+      <c r="M13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
-    <row r="14" ht="48" customHeight="1" spans="1:16">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
+    <row r="14" ht="73.5" customHeight="1" spans="1:16">
+      <c r="A14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="E14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
+      <c r="I14" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
+      <c r="M14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>27</v>
+      </c>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
+    </row>
+    <row r="15" ht="73.5" customHeight="1" spans="1:16">
+      <c r="A15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+    </row>
+    <row r="16" ht="73.5" customHeight="1" spans="1:16">
+      <c r="A16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
     </row>
     <row r="17" ht="21" customHeight="1" spans="1:13">
       <c r="A17" s="5" t="s">

</xml_diff>